<commit_message>
Fix risk math and rebuild the employer-facing models.
Correct the workbook cash-flow and portfolio-risk formulas, align Sharpe and credit ratings with the stated definitions, and add tested market-risk and loan-book analytics behind one dark theme.

Co-authored-by: Par Bahrae <githubproproject@proton.me>
</commit_message>
<xml_diff>
--- a/Advanced_Financial_Models.xlsx
+++ b/Advanced_Financial_Models.xlsx
@@ -349,13 +349,13 @@
     <t xml:space="preserve">Operating Expenses</t>
   </si>
   <si>
-    <t xml:space="preserve">  Salaries</t>
+    <t xml:space="preserve">  Salaries (included in operating expenses)</t>
   </si>
   <si>
     <t xml:space="preserve">  Rent</t>
   </si>
   <si>
-    <t xml:space="preserve">  Marketing</t>
+    <t xml:space="preserve">  Marketing (memo, not a separate cash outflow)</t>
   </si>
   <si>
     <t xml:space="preserve">Loan Payment</t>
@@ -859,7 +859,7 @@
     <t xml:space="preserve">Portfolio Expected Return</t>
   </si>
   <si>
-    <t xml:space="preserve">Portfolio Risk (Weighted Std Dev)</t>
+    <t xml:space="preserve">Portfolio Risk (zero correlation)</t>
   </si>
   <si>
     <t xml:space="preserve">Sharpe Ratio</t>
@@ -4714,47 +4714,47 @@
       </c>
       <c r="C15" s="15" t="n">
         <f aca="false">B28</f>
-        <v>-128000</v>
+        <v>77000</v>
       </c>
       <c r="D15" s="15" t="n">
         <f aca="false">C28</f>
-        <v>-118000</v>
+        <v>91000</v>
       </c>
       <c r="E15" s="15" t="n">
         <f aca="false">D28</f>
-        <v>-123250</v>
+        <v>122100</v>
       </c>
       <c r="F15" s="15" t="n">
         <f aca="false">E28</f>
-        <v>-143762.5</v>
+        <v>155405</v>
       </c>
       <c r="G15" s="15" t="n">
         <f aca="false">F28</f>
-        <v>-134550.625</v>
+        <v>176025.25</v>
       </c>
       <c r="H15" s="15" t="n">
         <f aca="false">G28</f>
-        <v>-140628.15625</v>
+        <v>214076.512500000012</v>
       </c>
       <c r="I15" s="15" t="n">
         <f aca="false">H28</f>
-        <v>-147009.5640625</v>
+        <v>254680.338125000038</v>
       </c>
       <c r="J15" s="15" t="n">
         <f aca="false">I28</f>
-        <v>-168710.042265625</v>
+        <v>297964.355031250045</v>
       </c>
       <c r="K15" s="15" t="n">
         <f aca="false">J28</f>
-        <v>-160745.544378906</v>
+        <v>329062.572782812582</v>
       </c>
       <c r="L15" s="15" t="n">
         <f aca="false">K28</f>
-        <v>-168132.821597852</v>
+        <v>378115.701421953214</v>
       </c>
       <c r="M15" s="15" t="n">
         <f aca="false">L28</f>
-        <v>-175889.462677744</v>
+        <v>430271.486493050877</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5130,20 +5130,20 @@
       <c r="A25" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B25" s="19" t="n">
+      <c r="B25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="19" t="n">
         <v>15000</v>
-      </c>
-      <c r="C25" s="15" t="n">
-        <v>0</v>
       </c>
       <c r="D25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E25" s="19" t="n">
+      <c r="E25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="19" t="n">
         <v>15000</v>
-      </c>
-      <c r="F25" s="15" t="n">
-        <v>0</v>
       </c>
       <c r="G25" s="15" t="n">
         <v>0</v>
@@ -5151,11 +5151,11 @@
       <c r="H25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="I25" s="19" t="n">
+      <c r="I25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="19" t="n">
         <v>15000</v>
-      </c>
-      <c r="J25" s="15" t="n">
-        <v>0</v>
       </c>
       <c r="K25" s="15" t="n">
         <v>0</v>
@@ -5172,52 +5172,52 @@
         <v>113</v>
       </c>
       <c r="B26" s="17" t="n">
-        <f aca="false">SUM(B20:B25)</f>
-        <v>128000</v>
+        <f aca="false">B20+B22+B24+B25</f>
+        <v>73000</v>
       </c>
       <c r="C26" s="17" t="n">
-        <f aca="false">SUM(C20:C25)</f>
-        <v>118000</v>
+        <f aca="false">C20+C22+C24+C25</f>
+        <v>91000</v>
       </c>
       <c r="D26" s="17" t="n">
-        <f aca="false">SUM(D20:D25)</f>
-        <v>123250</v>
+        <f aca="false">D20+D22+D24+D25</f>
+        <v>79150</v>
       </c>
       <c r="E26" s="17" t="n">
-        <f aca="false">SUM(E20:E25)</f>
-        <v>143762.5</v>
+        <f aca="false">E20+E22+E24+E25</f>
+        <v>82457.5</v>
       </c>
       <c r="F26" s="17" t="n">
-        <f aca="false">SUM(F20:F25)</f>
-        <v>134550.625</v>
+        <f aca="false">F20+F22+F24+F25</f>
+        <v>100930.375000000015</v>
       </c>
       <c r="G26" s="17" t="n">
-        <f aca="false">SUM(G20:G25)</f>
-        <v>140628.15625</v>
+        <f aca="false">G20+G22+G24+G25</f>
+        <v>89576.893750000017</v>
       </c>
       <c r="H26" s="17" t="n">
-        <f aca="false">SUM(H20:H25)</f>
-        <v>147009.5640625</v>
+        <f aca="false">H20+H22+H24+H25</f>
+        <v>93405.738437500026</v>
       </c>
       <c r="I26" s="17" t="n">
-        <f aca="false">SUM(I20:I25)</f>
-        <v>168710.042265625</v>
+        <f aca="false">I20+I22+I24+I25</f>
+        <v>97426.025359375039</v>
       </c>
       <c r="J26" s="17" t="n">
-        <f aca="false">SUM(J20:J25)</f>
-        <v>160745.544378906</v>
+        <f aca="false">J20+J22+J24+J25</f>
+        <v>116647.326627343791</v>
       </c>
       <c r="K26" s="17" t="n">
-        <f aca="false">SUM(K20:K25)</f>
-        <v>168132.821597852</v>
+        <f aca="false">K20+K22+K24+K25</f>
+        <v>106079.692958710963</v>
       </c>
       <c r="L26" s="17" t="n">
-        <f aca="false">SUM(L20:L25)</f>
-        <v>175889.462677744</v>
+        <f aca="false">L20+L22+L24+L25</f>
+        <v>110733.67760664651</v>
       </c>
       <c r="M26" s="17" t="n">
-        <f aca="false">SUM(M20:M25)</f>
-        <v>184033.935811631</v>
+        <f aca="false">M20+M22+M24+M25</f>
+        <v>115620.361486978843</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5225,52 +5225,52 @@
         <v>114</v>
       </c>
       <c r="B27" s="21" t="n">
-        <f aca="false">B19-B26</f>
-        <v>-128000</v>
+        <f aca="false">B18-B26</f>
+        <v>27000</v>
       </c>
       <c r="C27" s="21" t="n">
-        <f aca="false">C19-C26</f>
-        <v>-118000</v>
+        <f aca="false">C18-C26</f>
+        <v>14000</v>
       </c>
       <c r="D27" s="21" t="n">
-        <f aca="false">D19-D26</f>
-        <v>-123250</v>
+        <f aca="false">D18-D26</f>
+        <v>31100</v>
       </c>
       <c r="E27" s="21" t="n">
-        <f aca="false">E19-E26</f>
-        <v>-143762.5</v>
+        <f aca="false">E18-E26</f>
+        <v>33305</v>
       </c>
       <c r="F27" s="21" t="n">
-        <f aca="false">F19-F26</f>
-        <v>-134550.625</v>
+        <f aca="false">F18-F26</f>
+        <v>20620.250000000015</v>
       </c>
       <c r="G27" s="21" t="n">
-        <f aca="false">G19-G26</f>
-        <v>-140628.15625</v>
+        <f aca="false">G18-G26</f>
+        <v>38051.262500000012</v>
       </c>
       <c r="H27" s="21" t="n">
-        <f aca="false">H19-H26</f>
-        <v>-147009.5640625</v>
+        <f aca="false">H18-H26</f>
+        <v>40603.825625000027</v>
       </c>
       <c r="I27" s="21" t="n">
-        <f aca="false">I19-I26</f>
-        <v>-168710.042265625</v>
+        <f aca="false">I18-I26</f>
+        <v>43284.016906250021</v>
       </c>
       <c r="J27" s="21" t="n">
-        <f aca="false">J19-J26</f>
-        <v>-160745.544378906</v>
+        <f aca="false">J18-J26</f>
+        <v>31098.217751562523</v>
       </c>
       <c r="K27" s="21" t="n">
-        <f aca="false">K19-K26</f>
-        <v>-168132.821597852</v>
+        <f aca="false">K18-K26</f>
+        <v>49053.128639140647</v>
       </c>
       <c r="L27" s="21" t="n">
-        <f aca="false">L19-L26</f>
-        <v>-175889.462677744</v>
+        <f aca="false">L18-L26</f>
+        <v>52155.785071097678</v>
       </c>
       <c r="M27" s="21" t="n">
-        <f aca="false">M19-M26</f>
-        <v>-184033.935811631</v>
+        <f aca="false">M18-M26</f>
+        <v>55413.574324652567</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5278,52 +5278,52 @@
         <v>115</v>
       </c>
       <c r="B28" s="21" t="n">
-        <f aca="false">B16+B27</f>
-        <v>-128000</v>
+        <f aca="false">B15+B27</f>
+        <v>77000</v>
       </c>
       <c r="C28" s="21" t="n">
-        <f aca="false">C16+C27</f>
-        <v>-118000</v>
+        <f aca="false">C15+C27</f>
+        <v>91000</v>
       </c>
       <c r="D28" s="21" t="n">
-        <f aca="false">D16+D27</f>
-        <v>-123250</v>
+        <f aca="false">D15+D27</f>
+        <v>122100</v>
       </c>
       <c r="E28" s="21" t="n">
-        <f aca="false">E16+E27</f>
-        <v>-143762.5</v>
+        <f aca="false">E15+E27</f>
+        <v>155405</v>
       </c>
       <c r="F28" s="21" t="n">
-        <f aca="false">F16+F27</f>
-        <v>-134550.625</v>
+        <f aca="false">F15+F27</f>
+        <v>176025.25</v>
       </c>
       <c r="G28" s="21" t="n">
-        <f aca="false">G16+G27</f>
-        <v>-140628.15625</v>
+        <f aca="false">G15+G27</f>
+        <v>214076.512500000012</v>
       </c>
       <c r="H28" s="21" t="n">
-        <f aca="false">H16+H27</f>
-        <v>-147009.5640625</v>
+        <f aca="false">H15+H27</f>
+        <v>254680.338125000038</v>
       </c>
       <c r="I28" s="21" t="n">
-        <f aca="false">I16+I27</f>
-        <v>-168710.042265625</v>
+        <f aca="false">I15+I27</f>
+        <v>297964.355031250045</v>
       </c>
       <c r="J28" s="21" t="n">
-        <f aca="false">J16+J27</f>
-        <v>-160745.544378906</v>
+        <f aca="false">J15+J27</f>
+        <v>329062.572782812582</v>
       </c>
       <c r="K28" s="21" t="n">
-        <f aca="false">K16+K27</f>
-        <v>-168132.821597852</v>
+        <f aca="false">K15+K27</f>
+        <v>378115.701421953214</v>
       </c>
       <c r="L28" s="21" t="n">
-        <f aca="false">L16+L27</f>
-        <v>-175889.462677744</v>
+        <f aca="false">L15+L27</f>
+        <v>430271.486493050877</v>
       </c>
       <c r="M28" s="21" t="n">
-        <f aca="false">M16+M27</f>
-        <v>-184033.935811631</v>
+        <f aca="false">M15+M27</f>
+        <v>485685.06081770343</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5336,8 +5336,8 @@
         <v>117</v>
       </c>
       <c r="B32" s="15" t="n">
-        <f aca="false">NPV($B$10,C27:M27)+B27</f>
-        <v>-1072529.51362276</v>
+        <f aca="false">NPV((1+$B$10)^(1/12)-1,B27:M27)</f>
+        <v>410751.17267488403</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="B33" s="22" t="n">
         <f aca="false">AVERAGE(B27:M27)</f>
-        <v>-149392.721003688</v>
+        <v>36307.088401475288</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5355,7 +5355,7 @@
       </c>
       <c r="B34" s="15" t="n">
         <f aca="false">MIN(B28:M28)</f>
-        <v>-184033.935811631</v>
+        <v>77000</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="B35" s="15" t="n">
         <f aca="false">MAX(B28:M28)</f>
-        <v>-118000</v>
+        <v>485685.06081770343</v>
       </c>
     </row>
   </sheetData>
@@ -7605,8 +7605,8 @@
         <v>278</v>
       </c>
       <c r="B21" s="29" t="n">
-        <f aca="false">SQRT(SUMPRODUCT(D11:D16,C11:C16,C11:C16))</f>
-        <v>0.146471840297035</v>
+        <f aca="false">SQRT(SUMPRODUCT(D11:D16,D11:D16,C11:C16,C11:C16))</f>
+        <v>0.068240017585</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7615,7 +7615,7 @@
       </c>
       <c r="B22" s="34" t="n">
         <f aca="false">(B20-$B$6)/B21</f>
-        <v>0.385056949415156</v>
+        <v>0.82649451152</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Correct workbook formulas so they match the tested models
Cash-flow totals now use revenue minus operating expenses, rent, the loan
payment, and CapEx, with the $15,000 items in months 2, 5, and 9. NPV
discounts every month at the equivalent monthly rate. Portfolio risk uses
the same zero-correlation expression as the scenario rows and the Python
baseline. User-guide figures and the two README images that showed the old
results are updated to the recalculated values.

Co-authored-by: Par Bahrae <githubproproject@proton.me>
</commit_message>
<xml_diff>
--- a/Advanced_Financial_Models.xlsx
+++ b/Advanced_Financial_Models.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="297">
   <si>
     <t xml:space="preserve">Advanced Financial Modeling &amp; Forecasting - User Guide</t>
   </si>
@@ -88,7 +88,7 @@
     <t xml:space="preserve">How to Use: Modify BLUE inputs in rows 5-10 to test different scenarios</t>
   </si>
   <si>
-    <t xml:space="preserve">Key Metrics: NPV and IRR calculations based on net cash flows</t>
+    <t xml:space="preserve">Key Metrics: NPV of monthly net cash flows at the monthly equivalent of the annual discount rate</t>
   </si>
   <si>
     <t xml:space="preserve">Model 2: Loan Risk Model</t>
@@ -112,7 +112,7 @@
     <t xml:space="preserve">  • Expected Loss (EL) = Exposure × PD × LGD</t>
   </si>
   <si>
-    <t xml:space="preserve">  • Pivot table analysis of high-risk loans</t>
+    <t xml:space="preserve">  • Portfolio summary of exposure, expected loss, and risk-rating counts</t>
   </si>
   <si>
     <t xml:space="preserve">  • What-If analysis for different LGD scenarios</t>
@@ -349,13 +349,13 @@
     <t xml:space="preserve">Operating Expenses</t>
   </si>
   <si>
-    <t xml:space="preserve">  Salaries</t>
+    <t xml:space="preserve">  Salaries (memo, inside OpEx)</t>
   </si>
   <si>
     <t xml:space="preserve">  Rent</t>
   </si>
   <si>
-    <t xml:space="preserve">  Marketing</t>
+    <t xml:space="preserve">  Marketing (memo, not deducted)</t>
   </si>
   <si>
     <t xml:space="preserve">Loan Payment</t>
@@ -379,6 +379,9 @@
     <t xml:space="preserve">NPV of Cash Flows</t>
   </si>
   <si>
+    <t xml:space="preserve">(monthly equivalent rate, end of each month)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Average Monthly Net Cash Flow</t>
   </si>
   <si>
@@ -415,6 +418,9 @@
     <t xml:space="preserve">Risk-Free Rate</t>
   </si>
   <si>
+    <t xml:space="preserve">(reference only; not used in expected loss)</t>
+  </si>
+  <si>
     <t xml:space="preserve">800-850</t>
   </si>
   <si>
@@ -859,7 +865,7 @@
     <t xml:space="preserve">Portfolio Expected Return</t>
   </si>
   <si>
-    <t xml:space="preserve">Portfolio Risk (Weighted Std Dev)</t>
+    <t xml:space="preserve">Portfolio Risk (Zero Correlation)</t>
   </si>
   <si>
     <t xml:space="preserve">Sharpe Ratio</t>
@@ -1500,7 +1506,7 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-128000</c:v>
+                  <c:v>77000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1604,7 +1610,7 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-118000</c:v>
+                  <c:v>91000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1708,7 +1714,7 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-123250</c:v>
+                  <c:v>122100</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1812,7 +1818,7 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-143762.5</c:v>
+                  <c:v>155405</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1916,7 +1922,7 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-134550.625</c:v>
+                  <c:v>176025.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2020,7 +2026,7 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-140628.15625</c:v>
+                  <c:v>214076.5125</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2124,7 +2130,7 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-147009.5640625</c:v>
+                  <c:v>254680.338125</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2228,7 +2234,7 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-168710.042265625</c:v>
+                  <c:v>297964.35503125</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2332,7 +2338,7 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-160745.544378906</c:v>
+                  <c:v>329062.572782813</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2436,7 +2442,7 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-168132.821597852</c:v>
+                  <c:v>378115.701421953</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2540,7 +2546,7 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-175889.462677744</c:v>
+                  <c:v>430271.486493051</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2644,7 +2650,7 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-184033.935811631</c:v>
+                  <c:v>485685.060817703</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2659,11 +2665,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="8387713"/>
-        <c:axId val="25696632"/>
+        <c:axId val="90796083"/>
+        <c:axId val="32446351"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="8387713"/>
+        <c:axId val="90796083"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2729,7 +2735,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25696632"/>
+        <c:crossAx val="32446351"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2737,7 +2743,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="25696632"/>
+        <c:axId val="32446351"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2813,7 +2819,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8387713"/>
+        <c:crossAx val="90796083"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2992,11 +2998,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="1886933"/>
-        <c:axId val="93245437"/>
+        <c:axId val="82727897"/>
+        <c:axId val="81374468"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1886933"/>
+        <c:axId val="82727897"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3028,7 +3034,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93245437"/>
+        <c:crossAx val="81374468"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3036,7 +3042,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="93245437"/>
+        <c:axId val="81374468"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3078,7 +3084,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1886933"/>
+        <c:crossAx val="82727897"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3682,11 +3688,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="24776398"/>
-        <c:axId val="13453463"/>
+        <c:axId val="19351611"/>
+        <c:axId val="82212191"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="24776398"/>
+        <c:axId val="19351611"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3718,7 +3724,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13453463"/>
+        <c:crossAx val="82212191"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3726,7 +3732,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="13453463"/>
+        <c:axId val="82212191"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3802,7 +3808,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24776398"/>
+        <c:crossAx val="19351611"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3865,9 +3871,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>324000</xdr:colOff>
+      <xdr:colOff>323640</xdr:colOff>
       <xdr:row>44</xdr:row>
-      <xdr:rowOff>2160</xdr:rowOff>
+      <xdr:rowOff>1800</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3875,8 +3881,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="4299480" y="5713560"/>
-        <a:ext cx="5398920" cy="2699280"/>
+        <a:off x="4880520" y="5713560"/>
+        <a:ext cx="6084360" cy="2698920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3900,9 +3906,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>253800</xdr:colOff>
+      <xdr:colOff>253440</xdr:colOff>
       <xdr:row>82</xdr:row>
-      <xdr:rowOff>1800</xdr:rowOff>
+      <xdr:rowOff>1440</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3910,8 +3916,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="3171960" y="12952800"/>
-        <a:ext cx="5398920" cy="2698560"/>
+        <a:off x="3600360" y="12952800"/>
+        <a:ext cx="6094440" cy="2698200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3935,9 +3941,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>506880</xdr:colOff>
+      <xdr:colOff>506520</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>2160</xdr:rowOff>
+      <xdr:rowOff>1800</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3945,8 +3951,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="7730640" y="1713600"/>
-        <a:ext cx="5398920" cy="2698560"/>
+        <a:off x="8775720" y="1713600"/>
+        <a:ext cx="6064200" cy="2698200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3965,9 +3971,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>506880</xdr:colOff>
+      <xdr:colOff>506520</xdr:colOff>
       <xdr:row>46</xdr:row>
-      <xdr:rowOff>1800</xdr:rowOff>
+      <xdr:rowOff>1440</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3975,8 +3981,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="7730640" y="6094800"/>
-        <a:ext cx="5398920" cy="2698560"/>
+        <a:off x="8775720" y="6094800"/>
+        <a:ext cx="6064200" cy="2698200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4170,7 +4176,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A77"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="100"/>
   </cols>
@@ -4537,7 +4543,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="1" width="12"/>
@@ -4714,47 +4720,47 @@
       </c>
       <c r="C15" s="15" t="n">
         <f aca="false">B28</f>
-        <v>-128000</v>
+        <v>77000</v>
       </c>
       <c r="D15" s="15" t="n">
         <f aca="false">C28</f>
-        <v>-118000</v>
+        <v>91000</v>
       </c>
       <c r="E15" s="15" t="n">
         <f aca="false">D28</f>
-        <v>-123250</v>
+        <v>122100</v>
       </c>
       <c r="F15" s="15" t="n">
         <f aca="false">E28</f>
-        <v>-143762.5</v>
+        <v>155405</v>
       </c>
       <c r="G15" s="15" t="n">
         <f aca="false">F28</f>
-        <v>-134550.625</v>
+        <v>176025.25</v>
       </c>
       <c r="H15" s="15" t="n">
         <f aca="false">G28</f>
-        <v>-140628.15625</v>
+        <v>214076.5125</v>
       </c>
       <c r="I15" s="15" t="n">
         <f aca="false">H28</f>
-        <v>-147009.5640625</v>
+        <v>254680.338125</v>
       </c>
       <c r="J15" s="15" t="n">
         <f aca="false">I28</f>
-        <v>-168710.042265625</v>
+        <v>297964.35503125</v>
       </c>
       <c r="K15" s="15" t="n">
         <f aca="false">J28</f>
-        <v>-160745.544378906</v>
+        <v>329062.572782813</v>
       </c>
       <c r="L15" s="15" t="n">
         <f aca="false">K28</f>
-        <v>-168132.821597852</v>
+        <v>378115.701421953</v>
       </c>
       <c r="M15" s="15" t="n">
         <f aca="false">L28</f>
-        <v>-175889.462677744</v>
+        <v>430271.486493051</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5131,19 +5137,19 @@
         <v>112</v>
       </c>
       <c r="B25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="19" t="n">
         <v>15000</v>
-      </c>
-      <c r="C25" s="15" t="n">
-        <v>0</v>
       </c>
       <c r="D25" s="15" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="19" t="n">
         <v>15000</v>
-      </c>
-      <c r="F25" s="15" t="n">
-        <v>0</v>
       </c>
       <c r="G25" s="15" t="n">
         <v>0</v>
@@ -5152,10 +5158,10 @@
         <v>0</v>
       </c>
       <c r="I25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="19" t="n">
         <v>15000</v>
-      </c>
-      <c r="J25" s="15" t="n">
-        <v>0</v>
       </c>
       <c r="K25" s="15" t="n">
         <v>0</v>
@@ -5172,52 +5178,52 @@
         <v>113</v>
       </c>
       <c r="B26" s="17" t="n">
-        <f aca="false">SUM(B20:B25)</f>
-        <v>128000</v>
+        <f aca="false">B20+B22+B24+B25</f>
+        <v>73000</v>
       </c>
       <c r="C26" s="17" t="n">
-        <f aca="false">SUM(C20:C25)</f>
-        <v>118000</v>
+        <f aca="false">C20+C22+C24+C25</f>
+        <v>91000</v>
       </c>
       <c r="D26" s="17" t="n">
-        <f aca="false">SUM(D20:D25)</f>
-        <v>123250</v>
+        <f aca="false">D20+D22+D24+D25</f>
+        <v>79150</v>
       </c>
       <c r="E26" s="17" t="n">
-        <f aca="false">SUM(E20:E25)</f>
-        <v>143762.5</v>
+        <f aca="false">E20+E22+E24+E25</f>
+        <v>82457.5</v>
       </c>
       <c r="F26" s="17" t="n">
-        <f aca="false">SUM(F20:F25)</f>
-        <v>134550.625</v>
+        <f aca="false">F20+F22+F24+F25</f>
+        <v>100930.375</v>
       </c>
       <c r="G26" s="17" t="n">
-        <f aca="false">SUM(G20:G25)</f>
-        <v>140628.15625</v>
+        <f aca="false">G20+G22+G24+G25</f>
+        <v>89576.89375</v>
       </c>
       <c r="H26" s="17" t="n">
-        <f aca="false">SUM(H20:H25)</f>
-        <v>147009.5640625</v>
+        <f aca="false">H20+H22+H24+H25</f>
+        <v>93405.7384375</v>
       </c>
       <c r="I26" s="17" t="n">
-        <f aca="false">SUM(I20:I25)</f>
-        <v>168710.042265625</v>
+        <f aca="false">I20+I22+I24+I25</f>
+        <v>97426.025359375</v>
       </c>
       <c r="J26" s="17" t="n">
-        <f aca="false">SUM(J20:J25)</f>
-        <v>160745.544378906</v>
+        <f aca="false">J20+J22+J24+J25</f>
+        <v>116647.326627344</v>
       </c>
       <c r="K26" s="17" t="n">
-        <f aca="false">SUM(K20:K25)</f>
-        <v>168132.821597852</v>
+        <f aca="false">K20+K22+K24+K25</f>
+        <v>106079.692958711</v>
       </c>
       <c r="L26" s="17" t="n">
-        <f aca="false">SUM(L20:L25)</f>
-        <v>175889.462677744</v>
+        <f aca="false">L20+L22+L24+L25</f>
+        <v>110733.677606647</v>
       </c>
       <c r="M26" s="17" t="n">
-        <f aca="false">SUM(M20:M25)</f>
-        <v>184033.935811631</v>
+        <f aca="false">M20+M22+M24+M25</f>
+        <v>115620.361486979</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5225,52 +5231,52 @@
         <v>114</v>
       </c>
       <c r="B27" s="21" t="n">
-        <f aca="false">B19-B26</f>
-        <v>-128000</v>
+        <f aca="false">B18-B26</f>
+        <v>27000</v>
       </c>
       <c r="C27" s="21" t="n">
-        <f aca="false">C19-C26</f>
-        <v>-118000</v>
+        <f aca="false">C18-C26</f>
+        <v>14000</v>
       </c>
       <c r="D27" s="21" t="n">
-        <f aca="false">D19-D26</f>
-        <v>-123250</v>
+        <f aca="false">D18-D26</f>
+        <v>31100</v>
       </c>
       <c r="E27" s="21" t="n">
-        <f aca="false">E19-E26</f>
-        <v>-143762.5</v>
+        <f aca="false">E18-E26</f>
+        <v>33305</v>
       </c>
       <c r="F27" s="21" t="n">
-        <f aca="false">F19-F26</f>
-        <v>-134550.625</v>
+        <f aca="false">F18-F26</f>
+        <v>20620.25</v>
       </c>
       <c r="G27" s="21" t="n">
-        <f aca="false">G19-G26</f>
-        <v>-140628.15625</v>
+        <f aca="false">G18-G26</f>
+        <v>38051.2625</v>
       </c>
       <c r="H27" s="21" t="n">
-        <f aca="false">H19-H26</f>
-        <v>-147009.5640625</v>
+        <f aca="false">H18-H26</f>
+        <v>40603.825625</v>
       </c>
       <c r="I27" s="21" t="n">
-        <f aca="false">I19-I26</f>
-        <v>-168710.042265625</v>
+        <f aca="false">I18-I26</f>
+        <v>43284.01690625</v>
       </c>
       <c r="J27" s="21" t="n">
-        <f aca="false">J19-J26</f>
-        <v>-160745.544378906</v>
+        <f aca="false">J18-J26</f>
+        <v>31098.2177515625</v>
       </c>
       <c r="K27" s="21" t="n">
-        <f aca="false">K19-K26</f>
-        <v>-168132.821597852</v>
+        <f aca="false">K18-K26</f>
+        <v>49053.1286391406</v>
       </c>
       <c r="L27" s="21" t="n">
-        <f aca="false">L19-L26</f>
-        <v>-175889.462677744</v>
+        <f aca="false">L18-L26</f>
+        <v>52155.7850710977</v>
       </c>
       <c r="M27" s="21" t="n">
-        <f aca="false">M19-M26</f>
-        <v>-184033.935811631</v>
+        <f aca="false">M18-M26</f>
+        <v>55413.5743246526</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5278,52 +5284,52 @@
         <v>115</v>
       </c>
       <c r="B28" s="21" t="n">
-        <f aca="false">B16+B27</f>
-        <v>-128000</v>
+        <f aca="false">B15+B27</f>
+        <v>77000</v>
       </c>
       <c r="C28" s="21" t="n">
-        <f aca="false">C16+C27</f>
-        <v>-118000</v>
+        <f aca="false">C15+C27</f>
+        <v>91000</v>
       </c>
       <c r="D28" s="21" t="n">
-        <f aca="false">D16+D27</f>
-        <v>-123250</v>
+        <f aca="false">D15+D27</f>
+        <v>122100</v>
       </c>
       <c r="E28" s="21" t="n">
-        <f aca="false">E16+E27</f>
-        <v>-143762.5</v>
+        <f aca="false">E15+E27</f>
+        <v>155405</v>
       </c>
       <c r="F28" s="21" t="n">
-        <f aca="false">F16+F27</f>
-        <v>-134550.625</v>
+        <f aca="false">F15+F27</f>
+        <v>176025.25</v>
       </c>
       <c r="G28" s="21" t="n">
-        <f aca="false">G16+G27</f>
-        <v>-140628.15625</v>
+        <f aca="false">G15+G27</f>
+        <v>214076.5125</v>
       </c>
       <c r="H28" s="21" t="n">
-        <f aca="false">H16+H27</f>
-        <v>-147009.5640625</v>
+        <f aca="false">H15+H27</f>
+        <v>254680.338125</v>
       </c>
       <c r="I28" s="21" t="n">
-        <f aca="false">I16+I27</f>
-        <v>-168710.042265625</v>
+        <f aca="false">I15+I27</f>
+        <v>297964.35503125</v>
       </c>
       <c r="J28" s="21" t="n">
-        <f aca="false">J16+J27</f>
-        <v>-160745.544378906</v>
+        <f aca="false">J15+J27</f>
+        <v>329062.572782813</v>
       </c>
       <c r="K28" s="21" t="n">
-        <f aca="false">K16+K27</f>
-        <v>-168132.821597852</v>
+        <f aca="false">K15+K27</f>
+        <v>378115.701421953</v>
       </c>
       <c r="L28" s="21" t="n">
-        <f aca="false">L16+L27</f>
-        <v>-175889.462677744</v>
+        <f aca="false">L15+L27</f>
+        <v>430271.486493051</v>
       </c>
       <c r="M28" s="21" t="n">
-        <f aca="false">M16+M27</f>
-        <v>-184033.935811631</v>
+        <f aca="false">M15+M27</f>
+        <v>485685.060817703</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5336,35 +5342,38 @@
         <v>117</v>
       </c>
       <c r="B32" s="15" t="n">
-        <f aca="false">NPV($B$10,C27:M27)+B27</f>
-        <v>-1072529.51362276</v>
+        <f aca="false">NPV((1+$B$10)^(1/12)-1,B27:M27)</f>
+        <v>410751.172674884</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B33" s="22" t="n">
         <f aca="false">AVERAGE(B27:M27)</f>
-        <v>-149392.721003688</v>
+        <v>36307.0884014753</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B34" s="15" t="n">
         <f aca="false">MIN(B28:M28)</f>
-        <v>-184033.935811631</v>
+        <v>77000</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B35" s="15" t="n">
         <f aca="false">MAX(B28:M28)</f>
-        <v>-118000</v>
+        <v>485685.060817703</v>
       </c>
     </row>
   </sheetData>
@@ -5396,7 +5405,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I77"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
@@ -5410,170 +5419,173 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E4" s="23"/>
       <c r="F4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B5" s="10" t="n">
         <v>0.45</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B6" s="11" t="n">
         <v>0.03</v>
       </c>
+      <c r="C6" s="1" t="s">
+        <v>131</v>
+      </c>
       <c r="D6" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>0.01</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D7" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>0.02</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D8" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>0.04</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D9" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E9" s="11" t="n">
         <v>0.08</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D10" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E10" s="11" t="n">
         <v>0.15</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D11" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E11" s="11" t="n">
         <v>0.25</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D12" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0.35</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D13" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E13" s="11" t="n">
         <v>0.5</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C17" s="8" t="n">
         <v>345243</v>
@@ -5604,10 +5616,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C18" s="8" t="n">
         <v>23112</v>
@@ -5638,10 +5650,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C19" s="8" t="n">
         <v>154194</v>
@@ -5672,10 +5684,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C20" s="8" t="n">
         <v>127026</v>
@@ -5706,10 +5718,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C21" s="8" t="n">
         <v>396123</v>
@@ -5740,10 +5752,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C22" s="8" t="n">
         <v>364785</v>
@@ -5774,10 +5786,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C23" s="8" t="n">
         <v>477759</v>
@@ -5808,10 +5820,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C24" s="8" t="n">
         <v>55580</v>
@@ -5842,10 +5854,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C25" s="8" t="n">
         <v>231208</v>
@@ -5876,10 +5888,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C26" s="8" t="n">
         <v>25622</v>
@@ -5910,10 +5922,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C27" s="8" t="n">
         <v>124629</v>
@@ -5944,10 +5956,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C28" s="8" t="n">
         <v>274951</v>
@@ -5978,10 +5990,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C29" s="8" t="n">
         <v>23912</v>
@@ -6012,10 +6024,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C30" s="8" t="n">
         <v>114248</v>
@@ -6046,10 +6058,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C31" s="8" t="n">
         <v>350726</v>
@@ -6080,10 +6092,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C32" s="8" t="n">
         <v>295706</v>
@@ -6114,10 +6126,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C33" s="8" t="n">
         <v>125574</v>
@@ -6148,10 +6160,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C34" s="8" t="n">
         <v>318944</v>
@@ -6182,10 +6194,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C35" s="8" t="n">
         <v>434374</v>
@@ -6216,10 +6228,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C36" s="8" t="n">
         <v>407833</v>
@@ -6250,10 +6262,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C37" s="8" t="n">
         <v>376026</v>
@@ -6284,10 +6296,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C38" s="8" t="n">
         <v>188389</v>
@@ -6318,10 +6330,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C39" s="8" t="n">
         <v>91516</v>
@@ -6352,10 +6364,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C40" s="8" t="n">
         <v>410290</v>
@@ -6386,10 +6398,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C41" s="8" t="n">
         <v>63587</v>
@@ -6420,10 +6432,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C42" s="8" t="n">
         <v>209191</v>
@@ -6454,10 +6466,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C43" s="8" t="n">
         <v>198208</v>
@@ -6488,10 +6500,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C44" s="8" t="n">
         <v>326526</v>
@@ -6522,10 +6534,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C45" s="8" t="n">
         <v>433167</v>
@@ -6556,10 +6568,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C46" s="8" t="n">
         <v>392589</v>
@@ -6590,10 +6602,10 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C47" s="8" t="n">
         <v>291137</v>
@@ -6624,10 +6636,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C48" s="8" t="n">
         <v>493548</v>
@@ -6658,10 +6670,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C49" s="8" t="n">
         <v>51313</v>
@@ -6692,10 +6704,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C50" s="8" t="n">
         <v>163709</v>
@@ -6726,10 +6738,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C51" s="8" t="n">
         <v>334282</v>
@@ -6760,10 +6772,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C52" s="8" t="n">
         <v>312698</v>
@@ -6794,10 +6806,10 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C53" s="8" t="n">
         <v>379398</v>
@@ -6828,10 +6840,10 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C54" s="8" t="n">
         <v>34025</v>
@@ -6862,10 +6874,10 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C55" s="8" t="n">
         <v>129484</v>
@@ -6896,10 +6908,10 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C56" s="8" t="n">
         <v>161722</v>
@@ -6930,10 +6942,10 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C57" s="8" t="n">
         <v>458432</v>
@@ -6964,10 +6976,10 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C58" s="8" t="n">
         <v>464286</v>
@@ -6998,10 +7010,10 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C59" s="8" t="n">
         <v>209295</v>
@@ -7032,10 +7044,10 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C60" s="8" t="n">
         <v>247717</v>
@@ -7066,10 +7078,10 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C61" s="8" t="n">
         <v>447314</v>
@@ -7100,10 +7112,10 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C62" s="8" t="n">
         <v>95277</v>
@@ -7134,10 +7146,10 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C63" s="8" t="n">
         <v>196264</v>
@@ -7168,10 +7180,10 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C64" s="8" t="n">
         <v>361364</v>
@@ -7202,10 +7214,10 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C65" s="8" t="n">
         <v>377955</v>
@@ -7236,10 +7248,10 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C66" s="8" t="n">
         <v>349757</v>
@@ -7270,13 +7282,13 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="23" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B69" s="23"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B70" s="28" t="n">
         <f aca="false">COUNTA(A17:A66)</f>
@@ -7285,7 +7297,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B71" s="15" t="n">
         <f aca="false">SUM(C17:C66)</f>
@@ -7294,7 +7306,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B72" s="15" t="n">
         <f aca="false">SUM(H17:H66)</f>
@@ -7303,7 +7315,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B73" s="29" t="n">
         <f aca="false">B72/B71</f>
@@ -7312,7 +7324,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B74" s="1" t="n">
         <f aca="false">COUNTIF(I17:I66,"High")</f>
@@ -7321,7 +7333,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B75" s="1" t="n">
         <f aca="false">COUNTIF(I17:I66,"Medium")</f>
@@ -7330,7 +7342,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B76" s="1" t="n">
         <f aca="false">COUNTIF(I17:I66,"Low")</f>
@@ -7339,7 +7351,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B77" s="30" t="n">
         <f aca="false">AVERAGE(D17:D66)</f>
@@ -7368,7 +7380,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J30"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
@@ -7379,22 +7391,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B5" s="31" t="n">
         <v>1000000</v>
@@ -7402,7 +7414,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B6" s="11" t="n">
         <v>0.03</v>
@@ -7410,7 +7422,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B7" s="25" t="n">
         <v>10</v>
@@ -7418,27 +7430,27 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B11" s="11" t="n">
         <v>0.1</v>
@@ -7460,7 +7472,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B12" s="11" t="n">
         <v>0.12</v>
@@ -7482,7 +7494,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B13" s="11" t="n">
         <v>0.09</v>
@@ -7504,7 +7516,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B14" s="11" t="n">
         <v>0.05</v>
@@ -7526,7 +7538,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B15" s="11" t="n">
         <v>0.08</v>
@@ -7548,7 +7560,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B16" s="11" t="n">
         <v>0.06</v>
@@ -7570,7 +7582,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D17" s="32" t="n">
         <f aca="false">SUM(D11:D16)</f>
@@ -7587,13 +7599,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B19" s="23"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B20" s="29" t="n">
         <f aca="false">SUMPRODUCT(B11:B16,D11:D16)</f>
@@ -7602,25 +7614,25 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B21" s="29" t="n">
-        <f aca="false">SQRT(SUMPRODUCT(D11:D16,C11:C16,C11:C16))</f>
-        <v>0.146471840297035</v>
+        <f aca="false">SQRT(SUMPRODUCT(D11:D16,D11:D16,C11:C16,C11:C16))</f>
+        <v>0.0682400175849919</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B22" s="34" t="n">
         <f aca="false">(B20-$B$6)/B21</f>
-        <v>0.385056949415156</v>
+        <v>0.826494511519647</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B23" s="27" t="n">
         <f aca="false">$B$5*(1+B20)^$B$7</f>
@@ -7629,7 +7641,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B24" s="27" t="n">
         <f aca="false">B23-$B$5</f>
@@ -7638,7 +7650,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="23" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B26" s="23"/>
       <c r="C26" s="23"/>
@@ -7648,39 +7660,39 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="35" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B27" s="35" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C27" s="35" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D27" s="35" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E27" s="35" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="F27" s="35" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="G27" s="35" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="H27" s="35" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="I27" s="35" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="J27" s="35" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B28" s="22" t="n">
         <v>0.2</v>
@@ -7715,7 +7727,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B29" s="22" t="n">
         <v>0.3</v>
@@ -7750,7 +7762,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B30" s="22" t="n">
         <v>0.45</v>

</xml_diff>

<commit_message>
Reject impossible compounding and stop annualizing short samples.
A return at or below -100% no longer compounds to a negative future value. The market-risk board keeps short samples in period units, scales the risk-free rate by the fraction of a year covered, and hides 95% VaR until there are 20 observations.

Co-authored-by: Par Bahrae <githubproproject@proton.me>
</commit_message>
<xml_diff>
--- a/Advanced_Financial_Models.xlsx
+++ b/Advanced_Financial_Models.xlsx
@@ -88,7 +88,7 @@
     <t xml:space="preserve">How to Use: Modify BLUE inputs in rows 5-10 to test different scenarios</t>
   </si>
   <si>
-    <t xml:space="preserve">Key Metrics: NPV and IRR calculations based on net cash flows</t>
+    <t xml:space="preserve">Key Metrics: NPV of net cash flows</t>
   </si>
   <si>
     <t xml:space="preserve">Model 2: Loan Risk Model</t>
@@ -142,7 +142,7 @@
     <t xml:space="preserve">  • Portfolio expected return calculation</t>
   </si>
   <si>
-    <t xml:space="preserve">  • Portfolio risk (weighted standard deviation)</t>
+    <t xml:space="preserve">  • Portfolio risk (zero-correlation volatility)</t>
   </si>
   <si>
     <t xml:space="preserve">  • Sharpe Ratio for risk-adjusted returns</t>
@@ -166,7 +166,7 @@
     <t xml:space="preserve">Cash Flow Model:</t>
   </si>
   <si>
-    <t xml:space="preserve">  • Discount rate: 10% for NPV calculation</t>
+    <t xml:space="preserve">  • Discount rate: 10% annual, NPV uses the equivalent monthly rate</t>
   </si>
   <si>
     <t xml:space="preserve">  • Revenue growth: 5% monthly</t>
@@ -202,7 +202,7 @@
     <t xml:space="preserve">Advanced Excel Techniques Demonstrated</t>
   </si>
   <si>
-    <t xml:space="preserve">✓ Dynamic formulas: SUMIFS, XLOOKUP, NPV, IRR, STDEV</t>
+    <t xml:space="preserve">✓ Dynamic formulas: SUMIFS, XLOOKUP, NPV, STDEV</t>
   </si>
   <si>
     <t xml:space="preserve">✓ Conditional formatting with formulas</t>

</xml_diff>